<commit_message>
Actualizacion archivos ajustes de parametros y datos lote
</commit_message>
<xml_diff>
--- a/Data/Data_lote.xlsx
+++ b/Data/Data_lote.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gamez\OneDrive - Universidad EIA\Biocontrol_modeling_project\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/53da3c3e90e89215/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A567C06C-5EF2-4148-BFF3-8AB21929679F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{C2EDCC77-65A0-411C-A637-48A6763BED23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B7ECF4E-A5D8-41F3-8E8C-262ED7648C0A}"/>
   <bookViews>
-    <workbookView xWindow="1780" yWindow="1780" windowWidth="14400" windowHeight="7270" xr2:uid="{2A670E28-4D85-4653-96F3-C9FF6BA9A053}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{2A670E28-4D85-4653-96F3-C9FF6BA9A053}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>time</t>
   </si>
@@ -46,6 +46,15 @@
   </si>
   <si>
     <t>product</t>
+  </si>
+  <si>
+    <t>biomass_std</t>
+  </si>
+  <si>
+    <t>substrate_std</t>
+  </si>
+  <si>
+    <t>product_std</t>
   </si>
 </sst>
 </file>
@@ -101,7 +110,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -397,10 +406,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D474DA0-CF09-4399-84FD-F457B98D2777}">
-  <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -413,117 +422,313 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2">
-        <v>4.5900000000000003E-2</v>
+        <v>0</v>
       </c>
       <c r="B2">
-        <v>1.0975999999999999</v>
+        <v>0.5071</v>
       </c>
       <c r="C2">
-        <v>84.694800000000001</v>
+        <v>81.891400000000004</v>
       </c>
       <c r="D2">
+        <v>9.0700000000000003E-2</v>
+      </c>
+      <c r="E2">
+        <v>0.54390000000000005</v>
+      </c>
+      <c r="F2">
+        <v>4.3878000000000004</v>
+      </c>
+      <c r="G2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>3.2014999999999998</v>
+      </c>
+      <c r="C3">
+        <v>80.662800000000004</v>
+      </c>
+      <c r="D3">
+        <v>2.8000000000000001E-2</v>
+      </c>
+      <c r="E3">
+        <v>0.60399999999999998</v>
+      </c>
+      <c r="F3">
+        <v>4.3029000000000002</v>
+      </c>
+      <c r="G3">
+        <v>0.10730000000000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>6.2782999999999998</v>
+      </c>
+      <c r="C4">
+        <v>75.878699999999995</v>
+      </c>
+      <c r="D4">
+        <v>0.58350000000000002</v>
+      </c>
+      <c r="E4">
+        <v>0.74270000000000003</v>
+      </c>
+      <c r="F4">
+        <v>4.1064999999999996</v>
+      </c>
+      <c r="G4">
+        <v>0.124</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>12.093299999999999</v>
+      </c>
+      <c r="C5">
+        <v>74.948599999999999</v>
+      </c>
+      <c r="D5">
+        <v>1.3865000000000001</v>
+      </c>
+      <c r="E5">
+        <v>1.0468</v>
+      </c>
+      <c r="F5">
+        <v>3.6738</v>
+      </c>
+      <c r="G5">
+        <v>0.161</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>27.250599999999999</v>
+      </c>
+      <c r="C6">
+        <v>52.059800000000003</v>
+      </c>
+      <c r="D6">
+        <v>3.2587000000000002</v>
+      </c>
+      <c r="E6">
+        <v>1.6276999999999999</v>
+      </c>
+      <c r="F6">
+        <v>2.8344999999999998</v>
+      </c>
+      <c r="G6">
+        <v>0.23269999999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>50.148099999999999</v>
+      </c>
+      <c r="C7">
+        <v>19.8325</v>
+      </c>
+      <c r="D7">
+        <v>4.7732999999999999</v>
+      </c>
+      <c r="E7">
+        <v>2.3506</v>
+      </c>
+      <c r="F7">
+        <v>1.7241</v>
+      </c>
+      <c r="G7">
+        <v>0.3276</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8">
+        <v>12</v>
+      </c>
+      <c r="B8">
+        <v>46.389800000000001</v>
+      </c>
+      <c r="C8">
+        <v>3.5895999999999999</v>
+      </c>
+      <c r="D8">
+        <v>6.2964000000000002</v>
+      </c>
+      <c r="E8">
+        <v>2.6088</v>
+      </c>
+      <c r="F8">
+        <v>1.1262000000000001</v>
+      </c>
+      <c r="G8">
+        <v>0.37869999999999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9">
+        <v>14</v>
+      </c>
+      <c r="B9">
+        <v>48.340299999999999</v>
+      </c>
+      <c r="C9">
+        <v>1.1626000000000001</v>
+      </c>
+      <c r="D9">
+        <v>6.93</v>
+      </c>
+      <c r="E9">
+        <v>2.4761000000000002</v>
+      </c>
+      <c r="F9">
+        <v>1.0165</v>
+      </c>
+      <c r="G9">
+        <v>0.3881</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10">
+        <v>16</v>
+      </c>
+      <c r="B10">
+        <v>47.541899999999998</v>
+      </c>
+      <c r="C10">
+        <v>1.5559000000000001</v>
+      </c>
+      <c r="D10">
+        <v>7.5926</v>
+      </c>
+      <c r="E10">
+        <v>2.2858999999999998</v>
+      </c>
+      <c r="F10">
+        <v>1.0024999999999999</v>
+      </c>
+      <c r="G10">
+        <v>0.38929999999999998</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11">
+        <v>18</v>
+      </c>
+      <c r="B11">
+        <v>38.327599999999997</v>
+      </c>
+      <c r="C11">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>3.0678999999999998</v>
-      </c>
-      <c r="B3">
-        <v>2.9054000000000002</v>
-      </c>
-      <c r="C3">
-        <v>85.770200000000003</v>
-      </c>
-      <c r="D3">
+      <c r="D11">
+        <v>7.1683000000000003</v>
+      </c>
+      <c r="E11">
+        <v>2.1061000000000001</v>
+      </c>
+      <c r="F11">
+        <v>1.0004</v>
+      </c>
+      <c r="G11">
+        <v>0.38940000000000002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12">
+        <v>20</v>
+      </c>
+      <c r="B12">
+        <v>34.764099999999999</v>
+      </c>
+      <c r="C12">
+        <v>1.1782999999999999</v>
+      </c>
+      <c r="D12">
+        <v>7.2378</v>
+      </c>
+      <c r="E12">
+        <v>1.9433</v>
+      </c>
+      <c r="F12">
+        <v>1.0001</v>
+      </c>
+      <c r="G12">
+        <v>0.38950000000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13">
+        <v>22</v>
+      </c>
+      <c r="B13">
+        <v>32.2515</v>
+      </c>
+      <c r="C13">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>4.9687000000000001</v>
-      </c>
-      <c r="B4">
-        <v>9.6579999999999995</v>
-      </c>
-      <c r="C4">
-        <v>86.122200000000007</v>
-      </c>
-      <c r="D4">
-        <v>0.1462</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>7.0064000000000002</v>
-      </c>
-      <c r="B5">
-        <v>25.375399999999999</v>
-      </c>
-      <c r="C5">
-        <v>69.460899999999995</v>
-      </c>
-      <c r="D5">
-        <v>1.0466</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6">
-        <v>8.0238999999999994</v>
-      </c>
-      <c r="B6">
-        <v>37.258400000000002</v>
-      </c>
-      <c r="C6">
-        <v>58.477899999999998</v>
-      </c>
-      <c r="D6">
-        <v>3.6004</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7">
-        <v>8.9921000000000006</v>
-      </c>
-      <c r="B7">
-        <v>38.165199999999999</v>
-      </c>
-      <c r="C7">
-        <v>46.580500000000001</v>
-      </c>
-      <c r="D7">
-        <v>4.141</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8">
-        <v>14.2887</v>
-      </c>
-      <c r="B8">
-        <v>37.578299999999999</v>
-      </c>
-      <c r="C8">
-        <v>18.371099999999998</v>
-      </c>
-      <c r="D8">
-        <v>6.6641000000000004</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9">
-        <v>24.0746</v>
-      </c>
-      <c r="B9">
-        <v>34.396500000000003</v>
-      </c>
-      <c r="C9">
-        <v>0.9214</v>
-      </c>
-      <c r="D9">
-        <v>8.4214000000000002</v>
+      <c r="D13">
+        <v>7.5049000000000001</v>
+      </c>
+      <c r="E13">
+        <v>1.7968999999999999</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13">
+        <v>0.38950000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14">
+        <v>24</v>
+      </c>
+      <c r="B14">
+        <v>31.6142</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <v>6.8943000000000003</v>
+      </c>
+      <c r="E14">
+        <v>1.6652</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>0.38950000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>